<commit_message>
2 new users and updated the code profiles
</commit_message>
<xml_diff>
--- a/post_survey_responses.xlsx
+++ b/post_survey_responses.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -891,6 +891,256 @@
       <c r="P7" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="F8" t="n">
+        <v>6.01</v>
+      </c>
+      <c r="G8" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="H8" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="I8" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="K8" t="n">
+        <v>8.779999999999999</v>
+      </c>
+      <c r="L8" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>The vibrations felt slower paced and faster paced. It was easier to distinguish the faster ones and fell if they were slowing down or speeding up.</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>7.65</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Yes, some of the vibrations or patterns started feeling familiar.</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Trying to focus on either hearing or feeling the pattern only was much more difficult than both at the same time. Feeling the pattern was more difficult.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="F9" t="n">
+        <v>8</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="H9" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="I9" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="J9" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="K9" t="n">
+        <v>8.69</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>The vibrations were sometimes stronger or weaker but some felt constant which overall made it more difficult to determine if the pitch rising or lowering compared to the audio.</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>6.07</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>I started to become familiar with the audio and some of the vibrations.</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Thev vibration only feedbakc was much more difficult for me but when paired with the audio I felt like it made much more sense.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="E10" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="H10" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="I10" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="J10" t="n">
+        <v>5.53</v>
+      </c>
+      <c r="K10" t="n">
+        <v>6.01</v>
+      </c>
+      <c r="L10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Either really fast paced vibrations where it was easy to identify changes in tempo or moderate vibrations where it was difficult to notice changes. Features I tried to distinguish were the rate at which the vibrations occurred (i.e compared start and end rates)</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>6.63</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>If there was a dramatic change, it was most noticeable by comparing the start and end frequencies. I found most readings fell on a scale, where either it would slow down quickly or vice versa.</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Since I knew I was working with about 7 different frequencies expressed through different methods, my brain would ocassionally blank and it became difficult to decipher the smaller changes.</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Great gadget!</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="E11" t="n">
+        <v>5.71</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="G11" t="n">
+        <v>5.77</v>
+      </c>
+      <c r="H11" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="I11" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="K11" t="n">
+        <v>6.36</v>
+      </c>
+      <c r="L11" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Much faster vibrations. I tried to distinguish the vibration patters because they were either really fast or would noticeably slow down.</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>I would rest my finger nail on the vibration motor to get a much better sense of feel for the rates.</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>The adhesive tape lost its grip at times and felt like it coming off due to sweat. This made it hard to feel the subtle change in vibrations at times.</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Great!</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
final 3 people for initial analysis
</commit_message>
<xml_diff>
--- a/post_survey_responses.xlsx
+++ b/post_survey_responses.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1141,6 +1141,136 @@
       <c r="Q11" t="inlineStr">
         <is>
           <t>Great!</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>8.06</v>
+      </c>
+      <c r="D12" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="E12" t="n">
+        <v>5.53</v>
+      </c>
+      <c r="F12" t="n">
+        <v>8.029999999999999</v>
+      </c>
+      <c r="G12" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I12" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="J12" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="K12" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="L12" t="n">
+        <v>6.01</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>I felt vibrations that increased and decreased in tempo. Some vibrations' amplitudes were also varying per impulse. I tried to distinguish the higher amplitude vibrations fromthe softer ones in order to recognize the tempo.</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>10</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>I started to recognize the different kinds of samples I would receive and related the vibrations to the audio-only samples with this in mind.</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Some samples felt like the tempo was changing in both directions at times.</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>8</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>6.93</v>
+      </c>
+      <c r="F13" t="n">
+        <v>9.050000000000001</v>
+      </c>
+      <c r="G13" t="n">
+        <v>6.07</v>
+      </c>
+      <c r="H13" t="n">
+        <v>3</v>
+      </c>
+      <c r="I13" t="n">
+        <v>8.06</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" t="n">
+        <v>8.449999999999999</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>I experiennced vibrations that increased and decreased in "pitch". It was very hard to recognize what this pitch was, and I tried to use the "thumpy-ness" of the vibrations to indicate how low it was (i.e. if the vibration felt super heavy, it was a low pitch, and if it felt pretty light, it was a high pitch).</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>During the last portion with the mixed vibration-only, audio-only, and both samples, I used the samples that had both feedbacks to learn what the vibrations felt like during the rising pitch and falling pitches, as I was able to use the audio to confidently determine which was which. Then when given a vibration-only sample, I was able to remember what the mixed sample was like and try to determine its pitch change from that.</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>It was difficult to figure out what pitch really was in the vibration-only tests.</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>If there could be an example given of what high pitch and low pitch vibrations felt like before the test began, that may have been helpful in detecting the variation of pitch during the experiment.</t>
         </is>
       </c>
     </row>

</xml_diff>